<commit_message>
Recherche produit : rapport final, unit economics, fournisseurs, demande de devis
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AEK9oTC8uDjQF8VgcsLqgR
</commit_message>
<xml_diff>
--- a/recherche-produit/scoring.xlsx
+++ b/recherche-produit/scoring.xlsx
@@ -7580,14 +7580,14 @@
         <v>13.2</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>1.45</v>
+        <v>1.66</v>
       </c>
       <c r="F2" s="3">
         <f>D2*E2</f>
         <v/>
       </c>
       <c r="G2" s="2" t="n">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="H2" s="3">
         <f>G2/1.2</f>
@@ -7613,10 +7613,10 @@
         <v>20</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="O2" s="2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="P2" s="2" t="n">
         <v>12</v>
@@ -7634,7 +7634,7 @@
       </c>
       <c r="T2" s="5" t="inlineStr">
         <is>
-          <t>Demande : seul mot-clé de la shortlist avec volume réel et pic de Noël en hausse (56→87, +55 % en 4 ans, Google Trends). Concurrence : ~410 pubs Meta actives, Amazon inondé à 15-27 € (Ravmix 19 759 avis) → CAC élevé. Import : NC 6302 39 90, 12 % (TARIC). Prix usine 15 $ FOB (Xinlan/Zhigeng, data/fournisseurs_taie.csv) ; KO au critère 3 sous 76 € TTC. Rachat : cadeau Noël + extensions (masque, chouchous).</t>
+          <t>Demande : seul mot-clé de la shortlist avec volume réel et pic de Noël en hausse (56→87, +55 % en 4 ans, Google Trends). Concurrence : ~410 pubs Meta actives, Amazon inondé à 15-27 € (Ravmix 19 759 avis) → CAC élevé. Import : NC 6302 39 90, 12 % (TARIC). Prix usine 15 $ FOB (Xinlan/Zhigeng, data/fournisseurs_taie.csv) ; Coût rendu complet 21,88 € (unit-economics.xlsx) → KO à 79 € (27,7 %), OK à 89 € (24,6 %), prix au-dessus du cœur DTC 55-72 €. Rachat : cadeau Noël + extensions (masque, chouchous).</t>
         </is>
       </c>
     </row>
@@ -7646,7 +7646,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Chapeau Panama toquilla tissé main</t>
+          <t>Chapeau Panama toquilla tissé main (ÉLIMINÉ après coût rendu complet)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -7655,10 +7655,10 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>22</v>
+        <v>24.65</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>1.25</v>
+        <v>1.7</v>
       </c>
       <c r="F3" s="3">
         <f>D3*E3</f>
@@ -7691,7 +7691,7 @@
         <v>14</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="O3" s="2" t="n">
         <v>16</v>
@@ -7712,7 +7712,7 @@
       </c>
       <c r="T3" s="5" t="inlineStr">
         <is>
-          <t>Demande : moyenne 12 (échelle lot 1), pics juin-juillet 33-43, stable/légère baisse. Concurrence : 2 pubs Meta actives (1 annonceur). Import : NC 6504 00 00, 0 % (droit tiers 0 % + préférence Équateur, TARIC). Saison courte, rachat faible.</t>
+          <t>Coût rendu complet 41,81 € pour 36 pièces (fret volumétrique, boîte, transitaire) → 30 % du TTC et marge 64 % : KO critères 1 et 3. Demande : moyenne 12 (échelle lot 1), pics juin-juillet 33-43, stable/légère baisse. Concurrence : 2 pubs Meta actives (1 annonceur). Import : NC 6504 00 00, 0 % (droit tiers 0 % + préférence Équateur, TARIC). Saison courte, rachat faible.</t>
         </is>
       </c>
     </row>
@@ -7724,7 +7724,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Kimono coton imprimé au bloc (Jaipur)</t>
+          <t>Kimono long coton imprimé au bloc (Jaipur)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -7733,17 +7733,17 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>7.5</v>
+        <v>5.72</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>1.35</v>
+        <v>2.38</v>
       </c>
       <c r="F4" s="3">
         <f>D4*E4</f>
         <v/>
       </c>
       <c r="G4" s="2" t="n">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="H4" s="3">
         <f>G4/1.2</f>
@@ -7766,19 +7766,19 @@
         <v/>
       </c>
       <c r="M4" s="2" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="O4" s="2" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="P4" s="2" t="n">
         <v>12</v>
       </c>
       <c r="Q4" s="2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="R4">
         <f>SUM(M4:Q4)</f>
@@ -7790,7 +7790,7 @@
       </c>
       <c r="T4" s="5" t="inlineStr">
         <is>
-          <t>Demande : « kimono femme » moyenne 40 mais requête générique en baisse (~-40 % sur 5 ans). Concurrence : ~31 pubs Meta. Import : NC 6208 91 00 19, 12 % tiers / 9,6 % SPG Inde (TARIC). Marge très élevée (coût rendu ~13 % du TTC).</t>
+          <t>Demande : « kimono femme » = plus gros volume de la shortlist (moy. 40 vs 20 pour la taie) ; générique -40 % mais sous-segments « kimono femme abaya » +120 %, « chic » +120 %, « coton » +80 %. Concurrence : ~31 pubs Meta, Amazon sans acteur premium (259 résultats, ≤186 avis). Coût rendu complet 13,62 € (unit-economics.xlsx). Import : NC 6208 91 00 19, 12 % tiers / 9,6 % SPG Inde (TARIC). Marge très élevée (coût rendu ~13 % du TTC).</t>
         </is>
       </c>
     </row>
@@ -8378,7 +8378,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Prix usine × coefficient (fret + droits + transitaire + assurance). Coefficient 1,25 si droit 0 %, 1,30-1,35 si droit 12 %. Détail exact par produit dans unit-economics.xlsx.</t>
+          <t>Top 3 : coefficient = coût rendu complet / prix usine, issu de unit-economics.xlsx (fret, assurance, droits, transitaire, tests, packaging). Autres : prix usine × coefficient (fret + droits + transitaire + assurance). Coefficient 1,25 si droit 0 %, 1,30-1,35 si droit 12 %. Détail exact par produit dans unit-economics.xlsx.</t>
         </is>
       </c>
     </row>

</xml_diff>